<commit_message>
feat(auth): implement user registration and login with JWT authentication
</commit_message>
<xml_diff>
--- a/Mission Task Mananger Api.xlsx
+++ b/Mission Task Mananger Api.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DraconShade\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DraconShade\Desktop\task-manager-api\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A68B37E1-EFF2-4CF7-9BB3-E1E5BE3F7F40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17259468-0FD7-41AA-9AD6-3C4BEA497B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -196,7 +196,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -213,6 +213,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -523,7 +526,7 @@
       <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="2"/>
+      <c r="C4" s="8"/>
       <c r="F4" s="4" t="s">
         <v>15</v>
       </c>

</xml_diff>

<commit_message>
feat(validation): implement request validation across auth and task modules
</commit_message>
<xml_diff>
--- a/Mission Task Mananger Api.xlsx
+++ b/Mission Task Mananger Api.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DraconShade\Desktop\task-manager-api\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17259468-0FD7-41AA-9AD6-3C4BEA497B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9820A16C-4DB5-40EE-8447-C650608C0AAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -539,7 +539,7 @@
       <c r="B5" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="2"/>
+      <c r="C5" s="8"/>
       <c r="F5" s="4" t="s">
         <v>16</v>
       </c>
@@ -552,7 +552,7 @@
       <c r="B6" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="2"/>
+      <c r="C6" s="8"/>
       <c r="F6" s="4" t="s">
         <v>17</v>
       </c>
@@ -565,7 +565,7 @@
       <c r="B7" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="2"/>
+      <c r="C7" s="8"/>
       <c r="F7" s="4" t="s">
         <v>18</v>
       </c>
@@ -575,7 +575,7 @@
       <c r="B8" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="2"/>
+      <c r="C8" s="8"/>
       <c r="F8" s="4" t="s">
         <v>19</v>
       </c>
@@ -585,7 +585,7 @@
       <c r="B9" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="2"/>
+      <c r="C9" s="8"/>
       <c r="F9" s="4" t="s">
         <v>20</v>
       </c>
@@ -595,7 +595,7 @@
       <c r="B10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="2"/>
+      <c r="C10" s="8"/>
       <c r="F10" s="4" t="s">
         <v>21</v>
       </c>
@@ -605,7 +605,7 @@
       <c r="B11" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="2"/>
+      <c r="C11" s="8"/>
       <c r="F11" s="4" t="s">
         <v>22</v>
       </c>
@@ -615,13 +615,13 @@
       <c r="B12" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="2"/>
+      <c r="C12" s="8"/>
     </row>
     <row r="13" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B13" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="2"/>
+      <c r="C13" s="8"/>
     </row>
     <row r="14" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B14" s="5" t="s">

</xml_diff>